<commit_message>
Fixed Capitalization errors, added auditee name filtering for curl commands
</commit_message>
<xml_diff>
--- a/input_results.xlsx
+++ b/input_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,20 +429,25 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>auditee_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>local_path</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>message</t>
         </is>
@@ -459,20 +464,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>City Of Decatur</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-CITY_OF_DECATUR-376001308-2023.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-CITY_OF_DECATUR-376001308-2023.docx</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_Of_Decatur-376001308-2023.docx</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2023/MDL-City_Of_Decatur-376001308-2023.docx</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -485,20 +495,25 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>City of New London</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_New_London_CT-066001880-2024.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2024/MDL-City_of_New_London_CT-066001880-2024.docx</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_New_London-066001880-2024.docx</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2024/MDL-City_of_New_London-066001880-2024.docx</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -511,20 +526,25 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>City of Oregon</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Catholic_Community_Services_of_the_Mid-Willamette_Valley-936002230-2023.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-Catholic_Community_Services_of_the_Mid-Willamette_Valley-936002230-2023.docx</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_Oregon-936002230-2023.docx</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2023/MDL-City_of_Oregon-936002230-2023.docx</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -537,20 +557,25 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>City of Webster Groves</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_Webster_Groves-436003996-2024.docx</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>http://localhost:8000/local/mdl/2024/MDL-City_of_Webster_Groves-436003996-2024.docx</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -563,20 +588,25 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>County of Mariposa</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-COUNTY_OF_MARIPOSA-946000880-2023.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-COUNTY_OF_MARIPOSA-946000880-2023.docx</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-County_of_Mariposa-946000880-2023.docx</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2023/MDL-County_of_Mariposa-946000880-2023.docx</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -589,20 +619,25 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>County of Washington New York</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-COUNTY_OF_WASHINGTON_NEW_YORK-146002635-2024.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2024/MDL-COUNTY_OF_WASHINGTON_NEW_YORK-146002635-2024.docx</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-County_of_Washington_New_York-146002635-2024.docx</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2024/MDL-County_of_Washington_New_York-146002635-2024.docx</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -615,20 +650,25 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Gallatin County</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-GALLATIN_COUNTY-816001363-2022.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2022/MDL-GALLATIN_COUNTY-816001363-2022.docx</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Gallatin_County-816001363-2022.docx</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2022/MDL-Gallatin_County-816001363-2022.docx</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -641,20 +681,25 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Presidio County</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Presidio_County_Texas-746001689-2023.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-Presidio_County_Texas-746001689-2023.docx</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Presidio_County-746001689-2023.docx</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2023/MDL-Presidio_County-746001689-2023.docx</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -667,20 +712,25 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Town of Blacksburg Virginia</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-TOWN_OF_BLACKSBURG_VIRGINIA-546001146-2024.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2024/MDL-TOWN_OF_BLACKSBURG_VIRGINIA-546001146-2024.docx</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Town_of_Blacksburg_Virginia-546001146-2024.docx</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2024/MDL-Town_of_Blacksburg_Virginia-546001146-2024.docx</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -693,20 +743,25 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Town of Charlton</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-TOWN_OF_CHARLTON-046001109-2024.docx</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2024/MDL-TOWN_OF_CHARLTON-046001109-2024.docx</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Town_of_Charlton-046001109-2024.docx</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>http://localhost:8000/local/mdl/2024/MDL-Town_of_Charlton-046001109-2024.docx</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>